<commit_message>
Stabilize interview multisource RAG baseline
</commit_message>
<xml_diff>
--- a/aiops-docs/tickets.xlsx
+++ b/aiops-docs/tickets.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,32 +484,96 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>INC-REDIS-009</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>order-service</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>redis_maxclients</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Promotion lookup retry loop exhausted Redis client slots</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Reduced retry burst and capped idle Redis pool after approval</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Loki redis timeout Prometheus 5xx connected_clients near maxclients</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>INC-MYSQL-014</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>payment-service</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>mysql_slow_query</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Slow SQL held MySQL connections and caused pool waiting</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Captured digest, added index after approval, observed P95 recovery</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>slow_queries=18 active_connections=188/200 pool_waiting=6</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>INC-MYSQL-021</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>payment-service</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>mysql_pool_waiting</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Checkout report query caused MySQL pool_waiting after release rc3</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Disabled report flag, reviewed EXPLAIN, then added covering index</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>deploy rc3 slow query digest payment_report_join_v3 pool_waiting=6</t>
         </is>
       </c>
     </row>
@@ -524,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -584,27 +648,81 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>payment-service</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>payment-api-2026.07.06-rc4</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-07-06T10:32:00Z</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Disabled checkout report feature flag and prepared index change</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Remediation after approval; not an automatically executed Agent action</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>order-service</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>order-api-2026.07.06-rc1</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>2026-07-06T09:10:00Z</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Raised Redis retry count in promotion lookup path</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Can amplify Redis maxclients pressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>order-service</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>order-api-2026.07.06-rc2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-07-06T10:28:00Z</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Reduced Redis retry count and idle pool retention</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Remediation after approval for maxclients pressure</t>
         </is>
       </c>
     </row>

</xml_diff>